<commit_message>
Nimba Program bot - version 0.19.8 update
В отчётах о продажах озон теперь добавлены данные себестоимости, маржи на 1 единицу и чистой прибыли.
</commit_message>
<xml_diff>
--- a/market_bot/База данных артикулов для выкупов и начислений.xlsx
+++ b/market_bot/База данных артикулов для выкупов и начислений.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Шаблоны програм (Базы данных)\База данных (выкупы и начисления)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0A5DAE-65DF-4B0B-8427-E2DA3507E4E5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2833B9E9-C2E0-4AD8-A28C-CCE070912B2A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Отдельно Озон Nimba" sheetId="6" r:id="rId1"/>
@@ -19,8 +19,9 @@
     <sheet name="Отдельно ВБ Nimba" sheetId="7" r:id="rId4"/>
     <sheet name="Отдельно ВБ Galioni" sheetId="8" r:id="rId5"/>
     <sheet name="Отдельно ВБ AGNIA" sheetId="10" r:id="rId6"/>
-    <sheet name="Шаблон_WB" sheetId="4" r:id="rId7"/>
+    <sheet name="Cебестоимость" sheetId="11" r:id="rId7"/>
     <sheet name="Шаблон_Ozon" sheetId="3" r:id="rId8"/>
+    <sheet name="Шаблон_WB" sheetId="4" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Отдельно Озон Nimba'!$A$1:$D$60</definedName>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="301">
   <si>
     <t>накидка синий хлопок</t>
   </si>
@@ -936,6 +937,9 @@
   </si>
   <si>
     <t>детск. туника.голубой152</t>
+  </si>
+  <si>
+    <t>Себестоимость</t>
   </si>
 </sst>
 </file>
@@ -5644,20 +5648,16 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1C81525-87B5-40FD-A761-0FAE8806B157}">
-  <dimension ref="A1:K110"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8772D5-82E5-48C4-80EE-F2082BD24751}">
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="35" style="6" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="6"/>
-    <col min="4" max="4" width="30.42578125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="26.85546875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>79</v>
       </c>
@@ -5665,15 +5665,10 @@
         <v>82</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -5681,13 +5676,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="5">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -5695,13 +5687,10 @@
         <v>3</v>
       </c>
       <c r="C3" s="5">
-        <v>1</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -5709,13 +5698,10 @@
         <v>5</v>
       </c>
       <c r="C4" s="5">
-        <v>2</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -5723,13 +5709,10 @@
         <v>7</v>
       </c>
       <c r="C5" s="5">
-        <v>2</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -5737,13 +5720,10 @@
         <v>9</v>
       </c>
       <c r="C6" s="5">
-        <v>3</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -5751,13 +5731,10 @@
         <v>11</v>
       </c>
       <c r="C7" s="5">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -5765,13 +5742,10 @@
         <v>13</v>
       </c>
       <c r="C8" s="5">
-        <v>4</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -5779,13 +5753,10 @@
         <v>15</v>
       </c>
       <c r="C9" s="5">
-        <v>4</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -5793,13 +5764,10 @@
         <v>17</v>
       </c>
       <c r="C10" s="5">
-        <v>5</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -5807,13 +5775,10 @@
         <v>19</v>
       </c>
       <c r="C11" s="5">
-        <v>6</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -5821,13 +5786,10 @@
         <v>21</v>
       </c>
       <c r="C12" s="5">
-        <v>6</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -5835,13 +5797,10 @@
         <v>23</v>
       </c>
       <c r="C13" s="5">
-        <v>7</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -5849,13 +5808,10 @@
         <v>25</v>
       </c>
       <c r="C14" s="5">
-        <v>7</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -5863,13 +5819,10 @@
         <v>27</v>
       </c>
       <c r="C15" s="5">
-        <v>8</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -5877,13 +5830,10 @@
         <v>29</v>
       </c>
       <c r="C16" s="5">
-        <v>8</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -5891,13 +5841,10 @@
         <v>31</v>
       </c>
       <c r="C17" s="5">
-        <v>9</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -5905,13 +5852,10 @@
         <v>33</v>
       </c>
       <c r="C18" s="5">
-        <v>9</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -5919,13 +5863,10 @@
         <v>35</v>
       </c>
       <c r="C19" s="5">
-        <v>10</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -5933,13 +5874,10 @@
         <v>37</v>
       </c>
       <c r="C20" s="5">
-        <v>10</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -5947,13 +5885,10 @@
         <v>39</v>
       </c>
       <c r="C21" s="5">
-        <v>11</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -5961,13 +5896,10 @@
         <v>41</v>
       </c>
       <c r="C22" s="5">
-        <v>11</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -5975,13 +5907,10 @@
         <v>43</v>
       </c>
       <c r="C23" s="5">
-        <v>12</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -5989,13 +5918,10 @@
         <v>45</v>
       </c>
       <c r="C24" s="5">
-        <v>12</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -6003,13 +5929,10 @@
         <v>47</v>
       </c>
       <c r="C25" s="5">
-        <v>13</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -6017,13 +5940,10 @@
         <v>49</v>
       </c>
       <c r="C26" s="5">
-        <v>13</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -6031,13 +5951,10 @@
         <v>51</v>
       </c>
       <c r="C27" s="5">
-        <v>14</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -6045,13 +5962,10 @@
         <v>53</v>
       </c>
       <c r="C28" s="5">
-        <v>14</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -6059,13 +5973,10 @@
         <v>55</v>
       </c>
       <c r="C29" s="5">
-        <v>15</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -6073,13 +5984,10 @@
         <v>56</v>
       </c>
       <c r="C30" s="5">
-        <v>15</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -6087,13 +5995,10 @@
         <v>58</v>
       </c>
       <c r="C31" s="5">
-        <v>16</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -6101,13 +6006,10 @@
         <v>60</v>
       </c>
       <c r="C32" s="5">
-        <v>16</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -6115,13 +6017,10 @@
         <v>62</v>
       </c>
       <c r="C33" s="5">
-        <v>17</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -6129,13 +6028,10 @@
         <v>64</v>
       </c>
       <c r="C34" s="5">
-        <v>17</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -6143,13 +6039,10 @@
         <v>66</v>
       </c>
       <c r="C35" s="5">
-        <v>18</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -6157,13 +6050,10 @@
         <v>68</v>
       </c>
       <c r="C36" s="5">
-        <v>18</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -6171,13 +6061,10 @@
         <v>69</v>
       </c>
       <c r="C37" s="5">
-        <v>18</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -6185,13 +6072,10 @@
         <v>71</v>
       </c>
       <c r="C38" s="5">
-        <v>19</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -6199,13 +6083,10 @@
         <v>72</v>
       </c>
       <c r="C39" s="5">
-        <v>19</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -6213,601 +6094,67 @@
         <v>74</v>
       </c>
       <c r="C40" s="5">
-        <v>19</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>75</v>
+        <v>238</v>
       </c>
       <c r="C41" s="5">
-        <v>20</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C42" s="5">
-        <v>20</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C43" s="5">
-        <v>21</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="5">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="5">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C44" s="5">
-        <v>21</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C45" s="5">
-        <v>21</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C46" s="5">
-        <v>22</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C47" s="5">
-        <v>22</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C48" s="5">
-        <v>23</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C49" s="5">
-        <v>23</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C50" s="5">
-        <v>24</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C51" s="5">
-        <v>24</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C52" s="5">
-        <v>25</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C53" s="12">
-        <v>25</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C54" s="12">
-        <v>25</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C55" s="5">
-        <v>25</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="56" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C56" s="5">
-        <v>25</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="57" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C57" s="5">
-        <v>26</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C58" s="12">
-        <v>26</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="59" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C59" s="12">
-        <v>26</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="60" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C60" s="5">
-        <v>26</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="61" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C61" s="5">
-        <v>26</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="62" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C62" s="5">
-        <v>27</v>
-      </c>
-      <c r="D62" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="63" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C63" s="12">
-        <v>27</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="64" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C64" s="12">
-        <v>27</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C65" s="5">
-        <v>27</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C66" s="5">
-        <v>27</v>
-      </c>
-      <c r="D66" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C67" s="5">
-        <v>28</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C68" s="12">
-        <v>28</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C69" s="12">
-        <v>28</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C70" s="5">
-        <v>28</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C71" s="5">
-        <v>28</v>
-      </c>
-      <c r="D71" s="5" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C72" s="5">
-        <v>29</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C73" s="12">
-        <v>29</v>
-      </c>
-      <c r="D73" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C74" s="12">
-        <v>29</v>
-      </c>
-      <c r="D74" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="75" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C75" s="5">
-        <v>29</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="76" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C76" s="5">
-        <v>29</v>
-      </c>
-      <c r="D76" s="5" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C77" s="5">
-        <v>30</v>
-      </c>
-      <c r="D77" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C78" s="12">
-        <v>30</v>
-      </c>
-      <c r="D78" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="79" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C79" s="12">
-        <v>30</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="80" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C80" s="5">
-        <v>30</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C81" s="5">
-        <v>30</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C82" s="5">
-        <v>31</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C83" s="12">
-        <v>31</v>
-      </c>
-      <c r="D83" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="84" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C84" s="12">
-        <v>31</v>
-      </c>
-      <c r="D84" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C85" s="5">
-        <v>31</v>
-      </c>
-      <c r="D85" s="5" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C86" s="5">
-        <v>31</v>
-      </c>
-      <c r="D86" s="5" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="87" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C87" s="5">
-        <v>32</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="88" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C88" s="5">
-        <v>32</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="89" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C89" s="5">
-        <v>33</v>
-      </c>
-      <c r="D89" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="90" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C90" s="5">
-        <v>33</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="91" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C91" s="5">
-        <v>34</v>
-      </c>
-      <c r="D91" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="92" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C92" s="5">
-        <v>34</v>
-      </c>
-      <c r="D92" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="93" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C93" s="5">
-        <v>35</v>
-      </c>
-      <c r="D93" s="5" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="94" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C94" s="5">
-        <v>35</v>
-      </c>
-      <c r="D94" s="5" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="95" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C95" s="5">
-        <v>36</v>
-      </c>
-      <c r="D95" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="96" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C96" s="5">
-        <v>36</v>
-      </c>
-      <c r="D96" s="5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="97" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C97" s="5">
-        <v>37</v>
-      </c>
-      <c r="D97" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C98" s="5">
-        <v>37</v>
-      </c>
-      <c r="D98" s="5" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="99" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C99" s="12">
-        <v>38</v>
-      </c>
-      <c r="D99" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="100" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C100" s="5">
-        <v>38</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="101" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C101" s="12">
-        <v>39</v>
-      </c>
-      <c r="D101" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="102" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C102" s="5">
-        <v>39</v>
-      </c>
-      <c r="D102" s="5" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="103" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C103" s="12">
-        <v>40</v>
-      </c>
-      <c r="D103" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="104" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C104" s="5">
-        <v>40</v>
-      </c>
-      <c r="D104" s="5" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="105" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C105" s="5">
-        <v>41</v>
-      </c>
-      <c r="D105" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="106" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C106" s="5">
-        <v>41</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="107" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C107" s="5">
-        <v>42</v>
-      </c>
-      <c r="D107" s="5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="108" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C108" s="5">
-        <v>42</v>
-      </c>
-      <c r="D108" s="5" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="109" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C109" s="5">
-        <v>43</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="110" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C110" s="5">
-        <v>43</v>
-      </c>
-      <c r="D110" s="5" t="s">
-        <v>188</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:D110">
-    <sortCondition ref="C2:C110"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="261" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7927,4 +7274,1172 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1C81525-87B5-40FD-A761-0FAE8806B157}">
+  <dimension ref="A1:K110"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="35" style="6" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="6"/>
+    <col min="4" max="4" width="30.42578125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="26.85546875" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5">
+        <v>2</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="5">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="5">
+        <v>4</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="5">
+        <v>4</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="5">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="5">
+        <v>6</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="5">
+        <v>6</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="5">
+        <v>7</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="5">
+        <v>7</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="5">
+        <v>8</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="5">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="5">
+        <v>9</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="5">
+        <v>9</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="5">
+        <v>10</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="5">
+        <v>10</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="5">
+        <v>11</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="5">
+        <v>11</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="5">
+        <v>12</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="5">
+        <v>12</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="5">
+        <v>13</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="5">
+        <v>13</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="5">
+        <v>14</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="5">
+        <v>14</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="5">
+        <v>15</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C30" s="5">
+        <v>15</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="5">
+        <v>16</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="5">
+        <v>16</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" s="5">
+        <v>17</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="5">
+        <v>17</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C35" s="5">
+        <v>18</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="5">
+        <v>18</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" s="5">
+        <v>18</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" s="5">
+        <v>19</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" s="5">
+        <v>19</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="5">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C40" s="5">
+        <v>19</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="5">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="5">
+        <v>20</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="5">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" s="5">
+        <v>20</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="5">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" s="5">
+        <v>21</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="5">
+        <v>21</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C45" s="5">
+        <v>21</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C46" s="5">
+        <v>22</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C47" s="5">
+        <v>22</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C48" s="5">
+        <v>23</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C49" s="5">
+        <v>23</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C50" s="5">
+        <v>24</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C51" s="5">
+        <v>24</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C52" s="5">
+        <v>25</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C53" s="12">
+        <v>25</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C54" s="12">
+        <v>25</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C55" s="5">
+        <v>25</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="56" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C56" s="5">
+        <v>25</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="57" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C57" s="5">
+        <v>26</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C58" s="12">
+        <v>26</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="59" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C59" s="12">
+        <v>26</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C60" s="5">
+        <v>26</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="61" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C61" s="5">
+        <v>26</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="62" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C62" s="5">
+        <v>27</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="63" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C63" s="12">
+        <v>27</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="64" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C64" s="12">
+        <v>27</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C65" s="5">
+        <v>27</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C66" s="5">
+        <v>27</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C67" s="5">
+        <v>28</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C68" s="12">
+        <v>28</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C69" s="12">
+        <v>28</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C70" s="5">
+        <v>28</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C71" s="5">
+        <v>28</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C72" s="5">
+        <v>29</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C73" s="12">
+        <v>29</v>
+      </c>
+      <c r="D73" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C74" s="12">
+        <v>29</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C75" s="5">
+        <v>29</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="76" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C76" s="5">
+        <v>29</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C77" s="5">
+        <v>30</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C78" s="12">
+        <v>30</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="79" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C79" s="12">
+        <v>30</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="80" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C80" s="5">
+        <v>30</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C81" s="5">
+        <v>30</v>
+      </c>
+      <c r="D81" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C82" s="5">
+        <v>31</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C83" s="12">
+        <v>31</v>
+      </c>
+      <c r="D83" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="84" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C84" s="12">
+        <v>31</v>
+      </c>
+      <c r="D84" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C85" s="5">
+        <v>31</v>
+      </c>
+      <c r="D85" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C86" s="5">
+        <v>31</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="87" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C87" s="5">
+        <v>32</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="88" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C88" s="5">
+        <v>32</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="89" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C89" s="5">
+        <v>33</v>
+      </c>
+      <c r="D89" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="90" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C90" s="5">
+        <v>33</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="91" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C91" s="5">
+        <v>34</v>
+      </c>
+      <c r="D91" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="92" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C92" s="5">
+        <v>34</v>
+      </c>
+      <c r="D92" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C93" s="5">
+        <v>35</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="94" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C94" s="5">
+        <v>35</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="95" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C95" s="5">
+        <v>36</v>
+      </c>
+      <c r="D95" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="96" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C96" s="5">
+        <v>36</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="97" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C97" s="5">
+        <v>37</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C98" s="5">
+        <v>37</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="99" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C99" s="12">
+        <v>38</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="100" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C100" s="5">
+        <v>38</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="101" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C101" s="12">
+        <v>39</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="102" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C102" s="5">
+        <v>39</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="103" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C103" s="12">
+        <v>40</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="104" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C104" s="5">
+        <v>40</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="105" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C105" s="5">
+        <v>41</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="106" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C106" s="5">
+        <v>41</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="107" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C107" s="5">
+        <v>42</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="108" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C108" s="5">
+        <v>42</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="109" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C109" s="5">
+        <v>43</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="110" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C110" s="5">
+        <v>43</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:D110">
+    <sortCondition ref="C2:C110"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Nimba Program bot - version 0.19.8.1
</commit_message>
<xml_diff>
--- a/market_bot/База данных артикулов для выкупов и начислений.xlsx
+++ b/market_bot/База данных артикулов для выкупов и начислений.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Шаблоны програм (Базы данных)\База данных (выкупы и начисления)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2833B9E9-C2E0-4AD8-A28C-CCE070912B2A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4302F83E-3DB3-42B6-9AA7-5F8DA1668780}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5676,7 +5676,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -5687,7 +5687,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -5698,7 +5698,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -5709,7 +5709,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -5720,7 +5720,7 @@
         <v>9</v>
       </c>
       <c r="C6" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -5731,7 +5731,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -5742,7 +5742,7 @@
         <v>13</v>
       </c>
       <c r="C8" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -5753,7 +5753,7 @@
         <v>15</v>
       </c>
       <c r="C9" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -5764,7 +5764,7 @@
         <v>17</v>
       </c>
       <c r="C10" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -5775,7 +5775,7 @@
         <v>19</v>
       </c>
       <c r="C11" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -5786,7 +5786,7 @@
         <v>21</v>
       </c>
       <c r="C12" s="5">
-        <v>573</v>
+        <v>603</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -5797,7 +5797,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -5808,7 +5808,7 @@
         <v>25</v>
       </c>
       <c r="C14" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -5819,7 +5819,7 @@
         <v>27</v>
       </c>
       <c r="C15" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -5830,7 +5830,7 @@
         <v>29</v>
       </c>
       <c r="C16" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -5841,7 +5841,7 @@
         <v>31</v>
       </c>
       <c r="C17" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -5852,7 +5852,7 @@
         <v>33</v>
       </c>
       <c r="C18" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -5863,7 +5863,7 @@
         <v>35</v>
       </c>
       <c r="C19" s="5">
-        <v>682</v>
+        <v>712</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -5874,7 +5874,7 @@
         <v>37</v>
       </c>
       <c r="C20" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -5885,7 +5885,7 @@
         <v>39</v>
       </c>
       <c r="C21" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -5896,7 +5896,7 @@
         <v>41</v>
       </c>
       <c r="C22" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -5907,7 +5907,7 @@
         <v>43</v>
       </c>
       <c r="C23" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -5918,7 +5918,7 @@
         <v>45</v>
       </c>
       <c r="C24" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -5929,7 +5929,7 @@
         <v>47</v>
       </c>
       <c r="C25" s="5">
-        <v>593</v>
+        <v>623</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -5940,7 +5940,7 @@
         <v>49</v>
       </c>
       <c r="C26" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -5951,7 +5951,7 @@
         <v>51</v>
       </c>
       <c r="C27" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -5962,7 +5962,7 @@
         <v>53</v>
       </c>
       <c r="C28" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -5973,7 +5973,7 @@
         <v>55</v>
       </c>
       <c r="C29" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -5984,7 +5984,7 @@
         <v>56</v>
       </c>
       <c r="C30" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -5995,7 +5995,7 @@
         <v>58</v>
       </c>
       <c r="C31" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -6006,7 +6006,7 @@
         <v>60</v>
       </c>
       <c r="C32" s="5">
-        <v>709</v>
+        <v>739</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -6017,7 +6017,7 @@
         <v>62</v>
       </c>
       <c r="C33" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -6028,7 +6028,7 @@
         <v>64</v>
       </c>
       <c r="C34" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -6039,7 +6039,7 @@
         <v>66</v>
       </c>
       <c r="C35" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -6050,7 +6050,7 @@
         <v>68</v>
       </c>
       <c r="C36" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -6061,7 +6061,7 @@
         <v>69</v>
       </c>
       <c r="C37" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -6072,7 +6072,7 @@
         <v>71</v>
       </c>
       <c r="C38" s="5">
-        <v>675</v>
+        <v>705</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -6083,7 +6083,7 @@
         <v>72</v>
       </c>
       <c r="C39" s="5">
-        <v>560</v>
+        <v>660</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -6094,7 +6094,7 @@
         <v>74</v>
       </c>
       <c r="C40" s="5">
-        <v>560</v>
+        <v>660</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -6105,7 +6105,7 @@
         <v>238</v>
       </c>
       <c r="C41" s="5">
-        <v>560</v>
+        <v>660</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -6116,7 +6116,7 @@
         <v>75</v>
       </c>
       <c r="C42" s="5">
-        <v>560</v>
+        <v>660</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -6127,7 +6127,7 @@
         <v>76</v>
       </c>
       <c r="C43" s="5">
-        <v>290</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -6138,7 +6138,7 @@
         <v>77</v>
       </c>
       <c r="C44" s="5">
-        <v>290</v>
+        <v>320</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -6149,7 +6149,7 @@
         <v>78</v>
       </c>
       <c r="C45" s="5">
-        <v>290</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>